<commit_message>
removed all old comments. - Replaced `read_csv_clean` with `read_table_clean` across multiple modules for consistency and improved data handling. - Introduced atomic write functions `_atomic_write_xlsx` and `_atomic_write_json` to ensure safe file writing and prevent data corruption. - Updated scenario and diagnostics file paths to follow a consistent naming convention. - Enhanced the `run_scenario` and `run_test_set` functions to handle diagnostics more effectively. - Removed deprecated `__init__.py` file from the Architectures directory. - Updated tests to reflect changes in file handling and ensure compatibility with new diagnostics structure. - Modified ground truth calculators to utilize the new reading function for better data integrity.
</commit_message>
<xml_diff>
--- a/Scenario Files/TestScenarios.xlsx
+++ b/Scenario Files/TestScenarios.xlsx
@@ -6421,7 +6421,7 @@
         <v>28</v>
       </c>
       <c r="K107" t="n">
-        <v>105</v>
+        <v>60</v>
       </c>
       <c r="L107" t="inlineStr">
         <is>
@@ -6477,7 +6477,7 @@
         <v>75</v>
       </c>
       <c r="K108" t="n">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="L108" t="inlineStr">
         <is>
@@ -6533,7 +6533,7 @@
         <v>78</v>
       </c>
       <c r="K109" t="n">
-        <v>130</v>
+        <v>60</v>
       </c>
       <c r="L109" t="inlineStr">
         <is>
@@ -6589,7 +6589,7 @@
         <v>28</v>
       </c>
       <c r="K110" t="n">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="L110" t="inlineStr">
         <is>
@@ -6645,7 +6645,7 @@
         <v>32</v>
       </c>
       <c r="K111" t="n">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="L111" t="inlineStr">
         <is>
@@ -6701,7 +6701,7 @@
         <v>30</v>
       </c>
       <c r="K112" t="n">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="L112" t="inlineStr">
         <is>
@@ -6757,7 +6757,7 @@
         <v>82</v>
       </c>
       <c r="K113" t="n">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="L113" t="inlineStr">
         <is>
@@ -6813,7 +6813,7 @@
         <v>20</v>
       </c>
       <c r="K114" t="n">
-        <v>135</v>
+        <v>60</v>
       </c>
       <c r="L114" t="inlineStr">
         <is>
@@ -6869,7 +6869,7 @@
         <v>30</v>
       </c>
       <c r="K115" t="n">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="L115" t="inlineStr">
         <is>
@@ -6925,7 +6925,7 @@
         <v>85</v>
       </c>
       <c r="K116" t="n">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="L116" t="inlineStr">
         <is>
@@ -6981,7 +6981,7 @@
         <v>15</v>
       </c>
       <c r="K117" t="n">
-        <v>135</v>
+        <v>60</v>
       </c>
       <c r="L117" t="inlineStr">
         <is>
@@ -7037,7 +7037,7 @@
         <v>78</v>
       </c>
       <c r="K118" t="n">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="L118" t="inlineStr">
         <is>
@@ -7093,7 +7093,7 @@
         <v>88</v>
       </c>
       <c r="K119" t="n">
-        <v>140</v>
+        <v>60</v>
       </c>
       <c r="L119" t="inlineStr">
         <is>
@@ -7149,7 +7149,7 @@
         <v>22</v>
       </c>
       <c r="K120" t="n">
-        <v>105</v>
+        <v>60</v>
       </c>
       <c r="L120" t="inlineStr">
         <is>
@@ -7205,7 +7205,7 @@
         <v>30</v>
       </c>
       <c r="K121" t="n">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="L121" t="inlineStr">
         <is>
@@ -7261,7 +7261,7 @@
         <v>55</v>
       </c>
       <c r="K122" t="n">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="L122" t="inlineStr">
         <is>
@@ -7317,7 +7317,7 @@
         <v>58</v>
       </c>
       <c r="K123" t="n">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="L123" t="inlineStr">
         <is>
@@ -7373,7 +7373,7 @@
         <v>65</v>
       </c>
       <c r="K124" t="n">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="L124" t="inlineStr">
         <is>
@@ -7429,7 +7429,7 @@
         <v>50</v>
       </c>
       <c r="K125" t="n">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="L125" t="inlineStr">
         <is>
@@ -7485,7 +7485,7 @@
         <v>72</v>
       </c>
       <c r="K126" t="n">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="L126" t="inlineStr">
         <is>
@@ -7541,7 +7541,7 @@
         <v>52</v>
       </c>
       <c r="K127" t="n">
-        <v>105</v>
+        <v>60</v>
       </c>
       <c r="L127" t="inlineStr">
         <is>
@@ -7597,7 +7597,7 @@
         <v>45</v>
       </c>
       <c r="K128" t="n">
-        <v>105</v>
+        <v>60</v>
       </c>
       <c r="L128" t="inlineStr">
         <is>
@@ -7653,7 +7653,7 @@
         <v>55</v>
       </c>
       <c r="K129" t="n">
-        <v>130</v>
+        <v>60</v>
       </c>
       <c r="L129" t="inlineStr">
         <is>
@@ -7709,7 +7709,7 @@
         <v>55</v>
       </c>
       <c r="K130" t="n">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="L130" t="inlineStr">
         <is>
@@ -7765,7 +7765,7 @@
         <v>60</v>
       </c>
       <c r="K131" t="n">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="L131" t="inlineStr">
         <is>
@@ -7821,7 +7821,7 @@
         <v>92</v>
       </c>
       <c r="K132" t="n">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="L132" t="inlineStr">
         <is>
@@ -7877,7 +7877,7 @@
         <v>42</v>
       </c>
       <c r="K133" t="n">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="L133" t="inlineStr">
         <is>
@@ -7933,7 +7933,7 @@
         <v>38</v>
       </c>
       <c r="K134" t="n">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="L134" t="inlineStr">
         <is>
@@ -7989,7 +7989,7 @@
         <v>55</v>
       </c>
       <c r="K135" t="n">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="L135" t="inlineStr">
         <is>
@@ -8045,7 +8045,7 @@
         <v>62</v>
       </c>
       <c r="K136" t="n">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="L136" t="inlineStr">
         <is>
@@ -8101,7 +8101,7 @@
         <v>50</v>
       </c>
       <c r="K137" t="n">
-        <v>105</v>
+        <v>60</v>
       </c>
       <c r="L137" t="inlineStr">
         <is>
@@ -8157,7 +8157,7 @@
         <v>58</v>
       </c>
       <c r="K138" t="n">
-        <v>135</v>
+        <v>60</v>
       </c>
       <c r="L138" t="inlineStr">
         <is>
@@ -8213,7 +8213,7 @@
         <v>55</v>
       </c>
       <c r="K139" t="n">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="L139" t="inlineStr">
         <is>
@@ -8269,7 +8269,7 @@
         <v>58</v>
       </c>
       <c r="K140" t="n">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="L140" t="inlineStr">
         <is>
@@ -8325,7 +8325,7 @@
         <v>5</v>
       </c>
       <c r="K141" t="n">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="L141" t="inlineStr">
         <is>
@@ -9607,7 +9607,7 @@
         <v>62</v>
       </c>
       <c r="K164" t="n">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="L164" t="inlineStr">
         <is>
@@ -9663,7 +9663,7 @@
         <v>75</v>
       </c>
       <c r="K165" t="n">
-        <v>115</v>
+        <v>60</v>
       </c>
       <c r="L165" t="inlineStr">
         <is>
@@ -9719,7 +9719,7 @@
         <v>55</v>
       </c>
       <c r="K166" t="n">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="L166" t="inlineStr">
         <is>
@@ -9775,7 +9775,7 @@
         <v>62</v>
       </c>
       <c r="K167" t="n">
-        <v>115</v>
+        <v>60</v>
       </c>
       <c r="L167" t="inlineStr">
         <is>
@@ -9831,7 +9831,7 @@
         <v>48</v>
       </c>
       <c r="K168" t="n">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="L168" t="inlineStr">
         <is>
@@ -9887,7 +9887,7 @@
         <v>70</v>
       </c>
       <c r="K169" t="n">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="L169" t="inlineStr">
         <is>
@@ -9943,7 +9943,7 @@
         <v>38</v>
       </c>
       <c r="K170" t="n">
-        <v>105</v>
+        <v>60</v>
       </c>
       <c r="L170" t="inlineStr">
         <is>
@@ -9999,7 +9999,7 @@
         <v>45</v>
       </c>
       <c r="K171" t="n">
-        <v>110</v>
+        <v>60</v>
       </c>
       <c r="L171" t="inlineStr">
         <is>
@@ -10055,7 +10055,7 @@
         <v>52</v>
       </c>
       <c r="K172" t="n">
-        <v>115</v>
+        <v>60</v>
       </c>
       <c r="L172" t="inlineStr">
         <is>
@@ -10111,7 +10111,7 @@
         <v>48</v>
       </c>
       <c r="K173" t="n">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="L173" t="inlineStr">
         <is>
@@ -10167,7 +10167,7 @@
         <v>35</v>
       </c>
       <c r="K174" t="n">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="L174" t="inlineStr">
         <is>
@@ -10223,7 +10223,7 @@
         <v>60</v>
       </c>
       <c r="K175" t="n">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="L175" t="inlineStr">
         <is>
@@ -10279,7 +10279,7 @@
         <v>42</v>
       </c>
       <c r="K176" t="n">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="L176" t="inlineStr">
         <is>

</xml_diff>